<commit_message>
DJI dome nose on C8, smooth outlets, real cables on all four, print/CAD downloads
</commit_message>
<xml_diff>
--- a/c8/downloads/C8/SkyG-Speed-180-BOM.xlsx
+++ b/c8/downloads/C8/SkyG-Speed-180-BOM.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Order list (BOM)'!$A$4:$J$71</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Printed parts'!$A$4:$F$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Printed parts'!$A$4:$F$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3628,7 +3628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3870,7 +3870,7 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>N0O-nose-dji-o4</t>
+          <t>N0OD-dome-ring</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -3879,24 +3879,24 @@
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>6.1</v>
+        <v>0.3</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>0.76</v>
+        <v>0.04</v>
       </c>
       <c r="E12" s="6" t="n">
         <v>2</v>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>0 %</t>
+          <t>15 %</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>F1-fuselage-front</t>
+          <t>N0O-nose-dji-o4</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -3905,10 +3905,10 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>19.3</v>
+        <v>6.1</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>2.4</v>
+        <v>0.77</v>
       </c>
       <c r="E13" s="4" t="n">
         <v>2</v>
@@ -3922,7 +3922,7 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>F2-fuselage-main</t>
+          <t>N0OD-nose-dji-o4-dome</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -3931,10 +3931,10 @@
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>14.3</v>
+        <v>4.5</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>1.82</v>
+        <v>0.73</v>
       </c>
       <c r="E14" s="6" t="n">
         <v>2</v>
@@ -3948,7 +3948,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>F3-tail-module</t>
+          <t>F1-fuselage-front</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -3957,10 +3957,10 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>6.5</v>
+        <v>18.4</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>0.77</v>
+        <v>2.28</v>
       </c>
       <c r="E15" s="4" t="n">
         <v>2</v>
@@ -3974,7 +3974,7 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>HF-front-hatch</t>
+          <t>F2-fuselage-main</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -3983,10 +3983,10 @@
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>3.2</v>
+        <v>14.3</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>1.15</v>
+        <v>1.82</v>
       </c>
       <c r="E16" s="6" t="n">
         <v>2</v>
@@ -4000,7 +4000,7 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>HG-gps-carrier</t>
+          <t>F3-tail-module</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -4009,24 +4009,24 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>0.7</v>
+        <v>6.5</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>0.2</v>
+        <v>0.77</v>
       </c>
       <c r="E17" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>15 %</t>
+          <t>0 %</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>WR-wing-right</t>
+          <t>HF-front-hatch</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -4035,24 +4035,24 @@
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>11</v>
+        <v>3.2</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>1.75</v>
+        <v>1.15</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>5 %</t>
+          <t>0 %</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>WL-wing-left</t>
+          <t>HG-gps-carrier</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -4061,24 +4061,24 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>11.6</v>
+        <v>0.7</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>1.78</v>
+        <v>0.2</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>5 %</t>
+          <t>15 %</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>AR-aileron-right</t>
+          <t>WR-wing-right</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
@@ -4087,10 +4087,10 @@
         </is>
       </c>
       <c r="C20" s="6" t="n">
-        <v>1.5</v>
+        <v>11</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>0.61</v>
+        <v>1.75</v>
       </c>
       <c r="E20" s="6" t="n">
         <v>1</v>
@@ -4104,7 +4104,7 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>AL-aileron-left</t>
+          <t>WL-wing-left</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -4113,10 +4113,10 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>1.3</v>
+        <v>11.6</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>0.55</v>
+        <v>1.78</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
@@ -4130,7 +4130,7 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>SR-stabilator-right</t>
+          <t>AR-aileron-right</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -4139,24 +4139,24 @@
         </is>
       </c>
       <c r="C22" s="6" t="n">
-        <v>2.2</v>
+        <v>1.5</v>
       </c>
       <c r="D22" s="6" t="n">
-        <v>0.42</v>
+        <v>0.61</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>10 %</t>
+          <t>5 %</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>SL-stabilator-left</t>
+          <t>AL-aileron-left</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -4165,95 +4165,147 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>2.1</v>
+        <v>1.3</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>0.42</v>
+        <v>0.55</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>10 %</t>
+          <t>5 %</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>M1-motor-plate</t>
+          <t>SR-stabilator-right</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>PETG-CF</t>
+          <t>ASA Aero</t>
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>3.1</v>
+        <v>2.2</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>0.12</v>
+        <v>0.42</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>40 %</t>
+          <t>10 %</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
+          <t>SL-stabilator-left</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>ASA Aero</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>M1-motor-plate</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>PETG-CF</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
           <t>FN-fin</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>ASA Aero</t>
         </is>
       </c>
-      <c r="C25" s="4" t="n">
+      <c r="C27" s="4" t="n">
         <v>6.2</v>
       </c>
-      <c r="D25" s="4" t="n">
+      <c r="D27" s="4" t="n">
         <v>1.05</v>
       </c>
-      <c r="E25" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="E27" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
         <is>
           <t>15 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>One aircraft (one aircraft with the N0M nose; N0P is an alternative part): 88.3 g, 13.7 h of printing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Print every part with supports OFF, in the orientation of the user manual (all parts pass the print audit, design/DFAM-RULES.md).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>One aircraft (one aircraft with the N0M nose; N0P is an alternative part): 87.4 g, 13.6 h of printing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Print every part with supports OFF, in the orientation of the user manual (all parts pass the print audit, design/DFAM-RULES.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>Only one camera nose is needed; the other noses (and their dome ring or VTX shelf) are options.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F25"/>
+  <autoFilter ref="A4:F27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>